<commit_message>
Add 13 more simulation subjects (48-60) to reach 37 total
- 13 new subjects: 9 PITCH + 4 ODOR (all male)
- Fixed gender on 5 existing subjects (female->male) for target 29M/8F
- Final split: PITCH=19, ODOR=18 (equal)
- Updated both Excel files with all 37 subjects
- GI: ALL=616, PITCH=465, ODOR=776

https://claude.ai/code/session_0161wLfZ9d5BE5V6VedT4whE
</commit_message>
<xml_diff>
--- a/Garner_Simulation_Summary.xlsx
+++ b/Garner_Simulation_Summary.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J53"/>
+  <dimension ref="A1:J66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -499,7 +499,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>N=24 | PITCH=10 | ODOR=14</t>
+          <t>N=37 | PITCH=19 | ODOR=18</t>
         </is>
       </c>
     </row>
@@ -570,31 +570,31 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>2335.7</v>
+        <v>2176.9</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>906.6</v>
+        <v>861.7</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>2948.3</v>
+        <v>2793.3</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>1260.7</v>
+        <v>1145.1</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>2543</v>
+        <v>2270.2</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>1044.2</v>
+        <v>996.8</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>612.6</v>
+        <v>616.4</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>-207.3</v>
+        <v>-93.3</v>
       </c>
     </row>
     <row r="7">
@@ -604,31 +604,31 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>1590.8</v>
+        <v>1537.6</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>698.2</v>
+        <v>553.3</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>1974.3</v>
+        <v>2002.7</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>907.5</v>
+        <v>725.6</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>1674.9</v>
+        <v>1531.4</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>748</v>
+        <v>591</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>383.5</v>
+        <v>465.1</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>-84.09999999999999</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="8">
@@ -638,31 +638,31 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>2867.7</v>
+        <v>2851.7</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>620.6</v>
+        <v>556.1</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>3644</v>
+        <v>3627.9</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>995.5</v>
+        <v>885</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>3163.1</v>
+        <v>3050</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>740.3</v>
+        <v>693.1</v>
       </c>
       <c r="I8" s="7" t="n">
-        <v>776.3</v>
+        <v>776.2</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>-295.4</v>
+        <v>-198.3</v>
       </c>
     </row>
     <row r="9"/>
@@ -738,28 +738,28 @@
         </is>
       </c>
       <c r="C13" s="5" t="n">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>2387.1</v>
+        <v>2208.7</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>973.8</v>
+        <v>923.7</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>2559.5</v>
+        <v>2474.2</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>1031.3</v>
+        <v>975.1</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>2140.5</v>
+        <v>2011.3</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>848.4</v>
+        <v>803</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>172.4</v>
+        <v>265.5</v>
       </c>
     </row>
     <row r="14">
@@ -774,28 +774,28 @@
         </is>
       </c>
       <c r="C14" s="5" t="n">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="D14" s="5" t="n">
-        <v>2286.5</v>
+        <v>2140.5</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>854.6</v>
+        <v>817.8</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>3297.2</v>
+        <v>3077.8</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>1500.4</v>
+        <v>1353.9</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>2956.7</v>
+        <v>2536.2</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>1270.5</v>
+        <v>1235.2</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>1010.7</v>
+        <v>937.3</v>
       </c>
     </row>
     <row r="15">
@@ -810,28 +810,28 @@
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>1594.1</v>
+        <v>1525</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>726.1</v>
+        <v>570.1</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>1717.4</v>
+        <v>1753.1</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>698.7</v>
+        <v>559.6</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>1449.4</v>
+        <v>1415</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>662.5</v>
+        <v>513.3</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>123.3</v>
+        <v>228.1</v>
       </c>
     </row>
     <row r="16">
@@ -846,28 +846,28 @@
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>1592.4</v>
+        <v>1542.3</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>684.7</v>
+        <v>555.8</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>2225.7</v>
+        <v>2239.6</v>
       </c>
       <c r="G16" s="6" t="n">
-        <v>1128.9</v>
+        <v>945.2</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>1909.5</v>
+        <v>1653.2</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>853.1</v>
+        <v>700.6</v>
       </c>
       <c r="J16" s="6" t="n">
-        <v>633.3</v>
+        <v>697.3</v>
       </c>
     </row>
     <row r="17">
@@ -882,28 +882,28 @@
         </is>
       </c>
       <c r="C17" s="7" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D17" s="7" t="n">
-        <v>2953.5</v>
+        <v>2930.5</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>695.4</v>
+        <v>623.3</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>3161</v>
+        <v>3235.3</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>780.3</v>
+        <v>698.1</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>2634.1</v>
+        <v>2640.8</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>583</v>
+        <v>519.1</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>207.5</v>
+        <v>304.8</v>
       </c>
     </row>
     <row r="18">
@@ -918,28 +918,28 @@
         </is>
       </c>
       <c r="C18" s="7" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D18" s="7" t="n">
-        <v>2782.3</v>
+        <v>2772</v>
       </c>
       <c r="E18" s="7" t="n">
-        <v>576.5</v>
+        <v>516.6</v>
       </c>
       <c r="F18" s="7" t="n">
-        <v>4062.6</v>
+        <v>3962.5</v>
       </c>
       <c r="G18" s="7" t="n">
-        <v>1259.7</v>
+        <v>1149.6</v>
       </c>
       <c r="H18" s="7" t="n">
-        <v>3704.8</v>
+        <v>3468.1</v>
       </c>
       <c r="I18" s="7" t="n">
-        <v>951.7</v>
+        <v>959.3</v>
       </c>
       <c r="J18" s="7" t="n">
-        <v>1280.3</v>
+        <v>1190.5</v>
       </c>
     </row>
     <row r="19"/>
@@ -990,19 +990,19 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="C23" s="5" t="n">
-        <v>89.2</v>
+        <v>91.2</v>
       </c>
       <c r="D23" s="5" t="n">
-        <v>89.90000000000001</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>91.5</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>90.3</v>
+        <v>92.09999999999999</v>
       </c>
     </row>
     <row r="24">
@@ -1012,19 +1012,19 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="C24" s="6" t="n">
-        <v>90.8</v>
+        <v>93</v>
       </c>
       <c r="D24" s="6" t="n">
-        <v>95.8</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="E24" s="6" t="n">
-        <v>94.2</v>
+        <v>95</v>
       </c>
       <c r="F24" s="6" t="n">
-        <v>93.09999999999999</v>
+        <v>94.40000000000001</v>
       </c>
     </row>
     <row r="25">
@@ -1034,19 +1034,19 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C25" s="7" t="n">
-        <v>88.09999999999999</v>
+        <v>89.3</v>
       </c>
       <c r="D25" s="7" t="n">
-        <v>85.7</v>
+        <v>88</v>
       </c>
       <c r="E25" s="7" t="n">
+        <v>90.7</v>
+      </c>
+      <c r="F25" s="7" t="n">
         <v>89.59999999999999</v>
-      </c>
-      <c r="F25" s="7" t="n">
-        <v>88.2</v>
       </c>
     </row>
     <row r="26"/>
@@ -1695,6 +1695,331 @@
         <v>-147</v>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="n">
+        <v>1241.5</v>
+      </c>
+      <c r="D54" s="6" t="n">
+        <v>1805.33</v>
+      </c>
+      <c r="E54" s="6" t="n">
+        <v>563.8</v>
+      </c>
+      <c r="F54" s="6" t="n">
+        <v>1118.32</v>
+      </c>
+      <c r="G54" s="6" t="n">
+        <v>123.2</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="7" t="n">
+        <v>49</v>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>ODOR</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="n">
+        <v>2993.26</v>
+      </c>
+      <c r="D55" s="7" t="n">
+        <v>3355.18</v>
+      </c>
+      <c r="E55" s="7" t="n">
+        <v>361.9</v>
+      </c>
+      <c r="F55" s="7" t="n">
+        <v>2558.83</v>
+      </c>
+      <c r="G55" s="7" t="n">
+        <v>434.4</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="n">
+        <v>1552.45</v>
+      </c>
+      <c r="D56" s="6" t="n">
+        <v>2301.42</v>
+      </c>
+      <c r="E56" s="6" t="n">
+        <v>749</v>
+      </c>
+      <c r="F56" s="6" t="n">
+        <v>1441.5</v>
+      </c>
+      <c r="G56" s="6" t="n">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="7" t="n">
+        <v>51</v>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>ODOR</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="n">
+        <v>3026.46</v>
+      </c>
+      <c r="D57" s="7" t="n">
+        <v>3685.75</v>
+      </c>
+      <c r="E57" s="7" t="n">
+        <v>659.3</v>
+      </c>
+      <c r="F57" s="7" t="n">
+        <v>3067.23</v>
+      </c>
+      <c r="G57" s="7" t="n">
+        <v>-40.8</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="n">
+        <v>52</v>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="n">
+        <v>1141.67</v>
+      </c>
+      <c r="D58" s="6" t="n">
+        <v>1405.17</v>
+      </c>
+      <c r="E58" s="6" t="n">
+        <v>263.5</v>
+      </c>
+      <c r="F58" s="6" t="n">
+        <v>1026.25</v>
+      </c>
+      <c r="G58" s="6" t="n">
+        <v>115.4</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="n">
+        <v>53</v>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="n">
+        <v>1830.83</v>
+      </c>
+      <c r="D59" s="6" t="n">
+        <v>2431.27</v>
+      </c>
+      <c r="E59" s="6" t="n">
+        <v>600.4</v>
+      </c>
+      <c r="F59" s="6" t="n">
+        <v>1657.17</v>
+      </c>
+      <c r="G59" s="6" t="n">
+        <v>173.7</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="7" t="n">
+        <v>54</v>
+      </c>
+      <c r="B60" s="7" t="inlineStr">
+        <is>
+          <t>ODOR</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="n">
+        <v>2741.4</v>
+      </c>
+      <c r="D60" s="7" t="n">
+        <v>4040.67</v>
+      </c>
+      <c r="E60" s="7" t="n">
+        <v>1299.3</v>
+      </c>
+      <c r="F60" s="7" t="n">
+        <v>2543.5</v>
+      </c>
+      <c r="G60" s="7" t="n">
+        <v>197.9</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="n">
+        <v>55</v>
+      </c>
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="n">
+        <v>1005.48</v>
+      </c>
+      <c r="D61" s="6" t="n">
+        <v>1463.92</v>
+      </c>
+      <c r="E61" s="6" t="n">
+        <v>458.4</v>
+      </c>
+      <c r="F61" s="6" t="n">
+        <v>916.48</v>
+      </c>
+      <c r="G61" s="6" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="n">
+        <v>56</v>
+      </c>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="n">
+        <v>1365.73</v>
+      </c>
+      <c r="D62" s="6" t="n">
+        <v>2061.36</v>
+      </c>
+      <c r="E62" s="6" t="n">
+        <v>695.6</v>
+      </c>
+      <c r="F62" s="6" t="n">
+        <v>1415.21</v>
+      </c>
+      <c r="G62" s="6" t="n">
+        <v>-49.5</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="7" t="n">
+        <v>57</v>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>ODOR</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="n">
+        <v>2422</v>
+      </c>
+      <c r="D63" s="7" t="n">
+        <v>3204.09</v>
+      </c>
+      <c r="E63" s="7" t="n">
+        <v>782.1</v>
+      </c>
+      <c r="F63" s="7" t="n">
+        <v>2447.09</v>
+      </c>
+      <c r="G63" s="7" t="n">
+        <v>-25.1</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="n">
+        <v>58</v>
+      </c>
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="n">
+        <v>1322.12</v>
+      </c>
+      <c r="D64" s="6" t="n">
+        <v>1663.17</v>
+      </c>
+      <c r="E64" s="6" t="n">
+        <v>341.1</v>
+      </c>
+      <c r="F64" s="6" t="n">
+        <v>1270.14</v>
+      </c>
+      <c r="G64" s="6" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="n">
+        <v>2156</v>
+      </c>
+      <c r="D65" s="6" t="n">
+        <v>2971</v>
+      </c>
+      <c r="E65" s="6" t="n">
+        <v>815</v>
+      </c>
+      <c r="F65" s="6" t="n">
+        <v>1890.7</v>
+      </c>
+      <c r="G65" s="6" t="n">
+        <v>265.3</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="n">
+        <v>60</v>
+      </c>
+      <c r="B66" s="6" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="C66" s="6" t="n">
+        <v>1689.71</v>
+      </c>
+      <c r="D66" s="6" t="n">
+        <v>2205.55</v>
+      </c>
+      <c r="E66" s="6" t="n">
+        <v>515.8</v>
+      </c>
+      <c r="F66" s="6" t="n">
+        <v>1611.62</v>
+      </c>
+      <c r="G66" s="6" t="n">
+        <v>78.09999999999999</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 2 more male simulation subjects (61-62), total 39
- S61: ODOR, age 27, GI=+996
- S62: PITCH, age 24, GI=+740
- Final: 39 subjects, PITCH=20 ODOR=19, 31M/8F
- Updated both Excel files

https://claude.ai/code/session_0161wLfZ9d5BE5V6VedT4whE
</commit_message>
<xml_diff>
--- a/Garner_Simulation_Summary.xlsx
+++ b/Garner_Simulation_Summary.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J66"/>
+  <dimension ref="A1:J68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -499,7 +499,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>N=37 | PITCH=19 | ODOR=18</t>
+          <t>N=39 | PITCH=20 | ODOR=19</t>
         </is>
       </c>
     </row>
@@ -570,31 +570,31 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>2176.9</v>
+        <v>2178.9</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>861.7</v>
+        <v>860.3</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>2793.3</v>
+        <v>2808.3</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>1145.1</v>
+        <v>1138</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>2270.2</v>
+        <v>2252.2</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>996.8</v>
+        <v>983.9</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>616.4</v>
+        <v>629.4</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>-93.3</v>
+        <v>-73.3</v>
       </c>
     </row>
     <row r="7">
@@ -604,31 +604,31 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>1537.6</v>
+        <v>1529.9</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>553.3</v>
+        <v>539.6</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>2002.7</v>
+        <v>2008.7</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>725.6</v>
+        <v>706.8</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>1531.4</v>
+        <v>1519.6</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>591</v>
+        <v>577.6</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>465.1</v>
+        <v>478.8</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>6.2</v>
+        <v>10.3</v>
       </c>
     </row>
     <row r="8">
@@ -638,31 +638,31 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>2851.7</v>
+        <v>2862.2</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>556.1</v>
+        <v>542.4</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>3627.9</v>
+        <v>3649.9</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>885</v>
+        <v>865.4</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>3050</v>
+        <v>3023.5</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>693.1</v>
+        <v>683.4</v>
       </c>
       <c r="I8" s="7" t="n">
-        <v>776.2</v>
+        <v>787.7</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>-198.3</v>
+        <v>-161.3</v>
       </c>
     </row>
     <row r="9"/>
@@ -738,28 +738,28 @@
         </is>
       </c>
       <c r="C13" s="5" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>2208.7</v>
+        <v>2210.9</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>923.7</v>
+        <v>924.9</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>2474.2</v>
+        <v>2498.7</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>975.1</v>
+        <v>989.9</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>2011.3</v>
+        <v>2009.3</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>803</v>
+        <v>793.9</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>265.5</v>
+        <v>287.8</v>
       </c>
     </row>
     <row r="14">
@@ -774,28 +774,28 @@
         </is>
       </c>
       <c r="C14" s="5" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D14" s="5" t="n">
-        <v>2140.5</v>
+        <v>2141.5</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>817.8</v>
+        <v>811.9</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>3077.8</v>
+        <v>3091.2</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>1353.9</v>
+        <v>1328.3</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>2536.2</v>
+        <v>2502.1</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>1235.2</v>
+        <v>1220.3</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>937.3</v>
+        <v>949.7</v>
       </c>
     </row>
     <row r="15">
@@ -810,28 +810,28 @@
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>1525</v>
+        <v>1514</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>570.1</v>
+        <v>557.1</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>1753.1</v>
+        <v>1756.4</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>559.6</v>
+        <v>544.8</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>1415</v>
+        <v>1412.5</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>513.3</v>
+        <v>499.7</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>228.1</v>
+        <v>242.4</v>
       </c>
     </row>
     <row r="16">
@@ -846,28 +846,28 @@
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>1542.3</v>
+        <v>1538.3</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>555.8</v>
+        <v>541.3</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>2239.6</v>
+        <v>2260.5</v>
       </c>
       <c r="G16" s="6" t="n">
-        <v>945.2</v>
+        <v>924.7</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>1653.2</v>
+        <v>1632.1</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>700.6</v>
+        <v>688.4</v>
       </c>
       <c r="J16" s="6" t="n">
-        <v>697.3</v>
+        <v>722.2</v>
       </c>
     </row>
     <row r="17">
@@ -882,28 +882,28 @@
         </is>
       </c>
       <c r="C17" s="7" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D17" s="7" t="n">
-        <v>2930.5</v>
+        <v>2944.5</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>623.3</v>
+        <v>608.8</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>3235.3</v>
+        <v>3280.2</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>698.1</v>
+        <v>706.1</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>2640.8</v>
+        <v>2637.5</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>519.1</v>
+        <v>504.7</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>304.8</v>
+        <v>335.7</v>
       </c>
     </row>
     <row r="18">
@@ -918,28 +918,28 @@
         </is>
       </c>
       <c r="C18" s="7" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D18" s="7" t="n">
-        <v>2772</v>
+        <v>2776.4</v>
       </c>
       <c r="E18" s="7" t="n">
-        <v>516.6</v>
+        <v>502.4</v>
       </c>
       <c r="F18" s="7" t="n">
-        <v>3962.5</v>
+        <v>3965.7</v>
       </c>
       <c r="G18" s="7" t="n">
-        <v>1149.6</v>
+        <v>1117.3</v>
       </c>
       <c r="H18" s="7" t="n">
-        <v>3468.1</v>
+        <v>3417.9</v>
       </c>
       <c r="I18" s="7" t="n">
-        <v>959.3</v>
+        <v>957.6</v>
       </c>
       <c r="J18" s="7" t="n">
-        <v>1190.5</v>
+        <v>1189.3</v>
       </c>
     </row>
     <row r="19"/>
@@ -990,19 +990,19 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C23" s="5" t="n">
-        <v>91.2</v>
+        <v>91.3</v>
       </c>
       <c r="D23" s="5" t="n">
         <v>92.09999999999999</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>92.90000000000001</v>
+        <v>93.2</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>92.09999999999999</v>
+        <v>92.2</v>
       </c>
     </row>
     <row r="24">
@@ -1012,19 +1012,19 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C24" s="6" t="n">
-        <v>93</v>
+        <v>93.3</v>
       </c>
       <c r="D24" s="6" t="n">
-        <v>96.09999999999999</v>
+        <v>95.8</v>
       </c>
       <c r="E24" s="6" t="n">
         <v>95</v>
       </c>
       <c r="F24" s="6" t="n">
-        <v>94.40000000000001</v>
+        <v>94.5</v>
       </c>
     </row>
     <row r="25">
@@ -1034,19 +1034,19 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C25" s="7" t="n">
         <v>89.3</v>
       </c>
       <c r="D25" s="7" t="n">
-        <v>88</v>
+        <v>88.2</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>90.7</v>
+        <v>91.2</v>
       </c>
       <c r="F25" s="7" t="n">
-        <v>89.59999999999999</v>
+        <v>89.8</v>
       </c>
     </row>
     <row r="26"/>
@@ -2020,6 +2020,56 @@
         <v>78.09999999999999</v>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" s="7" t="n">
+        <v>61</v>
+      </c>
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>ODOR</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="n">
+        <v>3050.38</v>
+      </c>
+      <c r="D67" s="7" t="n">
+        <v>4046.18</v>
+      </c>
+      <c r="E67" s="7" t="n">
+        <v>995.8</v>
+      </c>
+      <c r="F67" s="7" t="n">
+        <v>2545.96</v>
+      </c>
+      <c r="G67" s="7" t="n">
+        <v>504.4</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="n">
+        <v>62</v>
+      </c>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="C68" s="6" t="n">
+        <v>1383.58</v>
+      </c>
+      <c r="D68" s="6" t="n">
+        <v>2123.55</v>
+      </c>
+      <c r="E68" s="6" t="n">
+        <v>740</v>
+      </c>
+      <c r="F68" s="6" t="n">
+        <v>1294.96</v>
+      </c>
+      <c r="G68" s="6" t="n">
+        <v>88.59999999999999</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 11 subjects (63-73), total 50 — balanced PITCH/ODOR 25/25
- 5F + 6M added (total: 37M/13F)
- 5 PITCH + 6 ODOR (total: 25/25 balanced)
- Ages 20-29, varied RT profiles
- Rebuilt all Excel files including statistical analysis

https://claude.ai/code/session_0161wLfZ9d5BE5V6VedT4whE
</commit_message>
<xml_diff>
--- a/Garner_Simulation_Summary.xlsx
+++ b/Garner_Simulation_Summary.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J68"/>
+  <dimension ref="A1:J79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -499,7 +499,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>N=39 | PITCH=20 | ODOR=19</t>
+          <t>N=50 | PITCH=25 | ODOR=25</t>
         </is>
       </c>
     </row>
@@ -570,31 +570,31 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>2178.9</v>
+        <v>2211.8</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>860.3</v>
+        <v>858.1</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>2808.3</v>
+        <v>2852.5</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>1138</v>
+        <v>1105.1</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>2252.2</v>
+        <v>2209</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>983.9</v>
+        <v>933.3</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>629.4</v>
+        <v>640.7</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>-73.3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="7">
@@ -604,31 +604,31 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>1529.9</v>
+        <v>1509.9</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>539.6</v>
+        <v>485</v>
       </c>
       <c r="E7" s="6" t="n">
         <v>2008.7</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>706.8</v>
+        <v>634.3</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>1519.6</v>
+        <v>1474.4</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>577.6</v>
+        <v>524.7</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>478.8</v>
+        <v>498.8</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>10.3</v>
+        <v>35.5</v>
       </c>
     </row>
     <row r="8">
@@ -638,31 +638,31 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>2862.2</v>
+        <v>2913.8</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>542.4</v>
+        <v>491.7</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>3649.9</v>
+        <v>3696.3</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>865.4</v>
+        <v>779.4</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>3023.5</v>
+        <v>2943.6</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>683.4</v>
+        <v>615.4</v>
       </c>
       <c r="I8" s="7" t="n">
-        <v>787.7</v>
+        <v>782.5</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>-161.3</v>
+        <v>-29.8</v>
       </c>
     </row>
     <row r="9"/>
@@ -738,28 +738,28 @@
         </is>
       </c>
       <c r="C13" s="5" t="n">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>2210.9</v>
+        <v>2236.4</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>924.9</v>
+        <v>898.3</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>2498.7</v>
+        <v>2548.2</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>989.9</v>
+        <v>976.3</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>2009.3</v>
+        <v>2014.6</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>793.9</v>
+        <v>769.5</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>287.8</v>
+        <v>311.8</v>
       </c>
     </row>
     <row r="14">
@@ -774,28 +774,28 @@
         </is>
       </c>
       <c r="C14" s="5" t="n">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="D14" s="5" t="n">
-        <v>2141.5</v>
+        <v>2183.9</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>811.9</v>
+        <v>842.9</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>3091.2</v>
+        <v>3133.2</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>1328.3</v>
+        <v>1296.2</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>2502.1</v>
+        <v>2408.3</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>1220.3</v>
+        <v>1146.6</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>949.7</v>
+        <v>949.3</v>
       </c>
     </row>
     <row r="15">
@@ -810,28 +810,28 @@
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>1514</v>
+        <v>1506</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>557.1</v>
+        <v>497.2</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>1756.4</v>
+        <v>1767.3</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>544.8</v>
+        <v>489.4</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>1412.5</v>
+        <v>1389.7</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>499.7</v>
+        <v>449.1</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>242.4</v>
+        <v>261.3</v>
       </c>
     </row>
     <row r="16">
@@ -846,28 +846,28 @@
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>1538.3</v>
+        <v>1506.9</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>541.3</v>
+        <v>491.4</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>2260.5</v>
+        <v>2243.7</v>
       </c>
       <c r="G16" s="6" t="n">
-        <v>924.7</v>
+        <v>828.6</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>1632.1</v>
+        <v>1562.7</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>688.4</v>
+        <v>631.9</v>
       </c>
       <c r="J16" s="6" t="n">
-        <v>722.2</v>
+        <v>736.8</v>
       </c>
     </row>
     <row r="17">
@@ -882,28 +882,28 @@
         </is>
       </c>
       <c r="C17" s="7" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="D17" s="7" t="n">
-        <v>2944.5</v>
+        <v>2966.9</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>608.8</v>
+        <v>537.3</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>3280.2</v>
+        <v>3329</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>706.1</v>
+        <v>660.3</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>2637.5</v>
+        <v>2639.4</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>504.7</v>
+        <v>440.4</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>335.7</v>
+        <v>362.1</v>
       </c>
     </row>
     <row r="18">
@@ -918,28 +918,28 @@
         </is>
       </c>
       <c r="C18" s="7" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="D18" s="7" t="n">
-        <v>2776.4</v>
+        <v>2860.8</v>
       </c>
       <c r="E18" s="7" t="n">
-        <v>502.4</v>
+        <v>504.2</v>
       </c>
       <c r="F18" s="7" t="n">
-        <v>3965.7</v>
+        <v>4022.7</v>
       </c>
       <c r="G18" s="7" t="n">
-        <v>1117.3</v>
+        <v>1046.4</v>
       </c>
       <c r="H18" s="7" t="n">
-        <v>3417.9</v>
+        <v>3254</v>
       </c>
       <c r="I18" s="7" t="n">
-        <v>957.6</v>
+        <v>891.5</v>
       </c>
       <c r="J18" s="7" t="n">
-        <v>1189.3</v>
+        <v>1161.9</v>
       </c>
     </row>
     <row r="19"/>
@@ -990,19 +990,19 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="C23" s="5" t="n">
-        <v>91.3</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="D23" s="5" t="n">
-        <v>92.09999999999999</v>
+        <v>92.2</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>93.2</v>
+        <v>93.3</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>92.2</v>
+        <v>92.40000000000001</v>
       </c>
     </row>
     <row r="24">
@@ -1012,16 +1012,16 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C24" s="6" t="n">
-        <v>93.3</v>
+        <v>93.8</v>
       </c>
       <c r="D24" s="6" t="n">
-        <v>95.8</v>
+        <v>95.7</v>
       </c>
       <c r="E24" s="6" t="n">
-        <v>95</v>
+        <v>94.5</v>
       </c>
       <c r="F24" s="6" t="n">
         <v>94.5</v>
@@ -1034,19 +1034,19 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="C25" s="7" t="n">
         <v>89.3</v>
       </c>
       <c r="D25" s="7" t="n">
-        <v>88.2</v>
+        <v>88.7</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>91.2</v>
+        <v>92.2</v>
       </c>
       <c r="F25" s="7" t="n">
-        <v>89.8</v>
+        <v>90.3</v>
       </c>
     </row>
     <row r="26"/>
@@ -2070,6 +2070,281 @@
         <v>88.59999999999999</v>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" s="7" t="n">
+        <v>63</v>
+      </c>
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>ODOR</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="n">
+        <v>2915.3</v>
+      </c>
+      <c r="D69" s="7" t="n">
+        <v>3863.18</v>
+      </c>
+      <c r="E69" s="7" t="n">
+        <v>947.9</v>
+      </c>
+      <c r="F69" s="7" t="n">
+        <v>2692.58</v>
+      </c>
+      <c r="G69" s="7" t="n">
+        <v>222.7</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="n">
+        <v>64</v>
+      </c>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="n">
+        <v>1658.83</v>
+      </c>
+      <c r="D70" s="6" t="n">
+        <v>2236.92</v>
+      </c>
+      <c r="E70" s="6" t="n">
+        <v>578.1</v>
+      </c>
+      <c r="F70" s="6" t="n">
+        <v>1398.61</v>
+      </c>
+      <c r="G70" s="6" t="n">
+        <v>260.2</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="7" t="n">
+        <v>65</v>
+      </c>
+      <c r="B71" s="7" t="inlineStr">
+        <is>
+          <t>ODOR</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="n">
+        <v>2825.3</v>
+      </c>
+      <c r="D71" s="7" t="n">
+        <v>4093.8</v>
+      </c>
+      <c r="E71" s="7" t="n">
+        <v>1268.5</v>
+      </c>
+      <c r="F71" s="7" t="n">
+        <v>2517.55</v>
+      </c>
+      <c r="G71" s="7" t="n">
+        <v>307.8</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="n">
+        <v>66</v>
+      </c>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="n">
+        <v>1313.54</v>
+      </c>
+      <c r="D72" s="6" t="n">
+        <v>1772</v>
+      </c>
+      <c r="E72" s="6" t="n">
+        <v>458.5</v>
+      </c>
+      <c r="F72" s="6" t="n">
+        <v>1219.52</v>
+      </c>
+      <c r="G72" s="6" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="7" t="n">
+        <v>67</v>
+      </c>
+      <c r="B73" s="7" t="inlineStr">
+        <is>
+          <t>ODOR</t>
+        </is>
+      </c>
+      <c r="C73" s="7" t="n">
+        <v>3382.75</v>
+      </c>
+      <c r="D73" s="7" t="n">
+        <v>4478.73</v>
+      </c>
+      <c r="E73" s="7" t="n">
+        <v>1096</v>
+      </c>
+      <c r="F73" s="7" t="n">
+        <v>3004.67</v>
+      </c>
+      <c r="G73" s="7" t="n">
+        <v>378.1</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="6" t="n">
+        <v>68</v>
+      </c>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="n">
+        <v>1402.71</v>
+      </c>
+      <c r="D74" s="6" t="n">
+        <v>2162.27</v>
+      </c>
+      <c r="E74" s="6" t="n">
+        <v>759.6</v>
+      </c>
+      <c r="F74" s="6" t="n">
+        <v>1449.5</v>
+      </c>
+      <c r="G74" s="6" t="n">
+        <v>-46.8</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="7" t="n">
+        <v>69</v>
+      </c>
+      <c r="B75" s="7" t="inlineStr">
+        <is>
+          <t>ODOR</t>
+        </is>
+      </c>
+      <c r="C75" s="7" t="n">
+        <v>2846.38</v>
+      </c>
+      <c r="D75" s="7" t="n">
+        <v>3253.27</v>
+      </c>
+      <c r="E75" s="7" t="n">
+        <v>406.9</v>
+      </c>
+      <c r="F75" s="7" t="n">
+        <v>2481.65</v>
+      </c>
+      <c r="G75" s="7" t="n">
+        <v>364.7</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="n">
+        <v>70</v>
+      </c>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="n">
+        <v>1422.87</v>
+      </c>
+      <c r="D76" s="6" t="n">
+        <v>2046</v>
+      </c>
+      <c r="E76" s="6" t="n">
+        <v>623.1</v>
+      </c>
+      <c r="F76" s="6" t="n">
+        <v>1247.74</v>
+      </c>
+      <c r="G76" s="6" t="n">
+        <v>175.1</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="7" t="n">
+        <v>71</v>
+      </c>
+      <c r="B77" s="7" t="inlineStr">
+        <is>
+          <t>ODOR</t>
+        </is>
+      </c>
+      <c r="C77" s="7" t="n">
+        <v>3204.29</v>
+      </c>
+      <c r="D77" s="7" t="n">
+        <v>3506.36</v>
+      </c>
+      <c r="E77" s="7" t="n">
+        <v>302.1</v>
+      </c>
+      <c r="F77" s="7" t="n">
+        <v>2771.14</v>
+      </c>
+      <c r="G77" s="7" t="n">
+        <v>433.2</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="7" t="n">
+        <v>72</v>
+      </c>
+      <c r="B78" s="7" t="inlineStr">
+        <is>
+          <t>ODOR</t>
+        </is>
+      </c>
+      <c r="C78" s="7" t="n">
+        <v>3288.55</v>
+      </c>
+      <c r="D78" s="7" t="n">
+        <v>3864.82</v>
+      </c>
+      <c r="E78" s="7" t="n">
+        <v>576.3</v>
+      </c>
+      <c r="F78" s="7" t="n">
+        <v>2676.65</v>
+      </c>
+      <c r="G78" s="7" t="n">
+        <v>611.9</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="6" t="n">
+        <v>73</v>
+      </c>
+      <c r="B79" s="6" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="C79" s="6" t="n">
+        <v>1352.71</v>
+      </c>
+      <c r="D79" s="6" t="n">
+        <v>1825.83</v>
+      </c>
+      <c r="E79" s="6" t="n">
+        <v>473.1</v>
+      </c>
+      <c r="F79" s="6" t="n">
+        <v>1152.45</v>
+      </c>
+      <c r="G79" s="6" t="n">
+        <v>200.3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 2 male subjects (74-75), total 52 — PITCH/ODOR 26/26
- S74: ODOR, age 23, GI=+1440
- S75: PITCH, age 26, GI=+719
- Updated all Excel files

https://claude.ai/code/session_0161wLfZ9d5BE5V6VedT4whE
</commit_message>
<xml_diff>
--- a/Garner_Simulation_Summary.xlsx
+++ b/Garner_Simulation_Summary.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J79"/>
+  <dimension ref="A1:J81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -499,7 +499,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>N=50 | PITCH=25 | ODOR=25</t>
+          <t>N=52 | PITCH=26 | ODOR=26</t>
         </is>
       </c>
     </row>
@@ -570,31 +570,31 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>2211.8</v>
+        <v>2209.3</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>858.1</v>
+        <v>847.6</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>2852.5</v>
+        <v>2866.8</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>1105.1</v>
+        <v>1099.6</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>2209</v>
+        <v>2208.3</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>933.3</v>
+        <v>924.8</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>640.7</v>
+        <v>657.5</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>2.8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -604,31 +604,31 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>1509.9</v>
+        <v>1514.2</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>485</v>
+        <v>475.7</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>2008.7</v>
+        <v>2021.5</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>634.3</v>
+        <v>624.9</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>1474.4</v>
+        <v>1475.6</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>524.7</v>
+        <v>514.1</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>498.8</v>
+        <v>507.3</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>35.5</v>
+        <v>38.6</v>
       </c>
     </row>
     <row r="8">
@@ -638,31 +638,31 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>2913.8</v>
+        <v>2904.3</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>491.7</v>
+        <v>484.2</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>3696.3</v>
+        <v>3712.2</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>779.4</v>
+        <v>768</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>2943.6</v>
+        <v>2941</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>615.4</v>
+        <v>603.2</v>
       </c>
       <c r="I8" s="7" t="n">
-        <v>782.5</v>
+        <v>807.9</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>-29.8</v>
+        <v>-36.7</v>
       </c>
     </row>
     <row r="9"/>
@@ -738,28 +738,28 @@
         </is>
       </c>
       <c r="C13" s="5" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>2236.4</v>
+        <v>2237</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>898.3</v>
+        <v>888.7</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>2548.2</v>
+        <v>2576.4</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>976.3</v>
+        <v>984.4</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>2014.6</v>
+        <v>2028.3</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>769.5</v>
+        <v>768.9</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>311.8</v>
+        <v>339.4</v>
       </c>
     </row>
     <row r="14">
@@ -774,28 +774,28 @@
         </is>
       </c>
       <c r="C14" s="5" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D14" s="5" t="n">
-        <v>2183.9</v>
+        <v>2179.4</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>842.9</v>
+        <v>831.7</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>3133.2</v>
+        <v>3131.1</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>1296.2</v>
+        <v>1279.3</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>2408.3</v>
+        <v>2393.4</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>1146.6</v>
+        <v>1134.7</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>949.3</v>
+        <v>951.7</v>
       </c>
     </row>
     <row r="15">
@@ -810,28 +810,28 @@
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>1506</v>
+        <v>1511.2</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>497.2</v>
+        <v>487.9</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>1767.3</v>
+        <v>1790.3</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>489.4</v>
+        <v>493.7</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>1389.7</v>
+        <v>1401.8</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>449.1</v>
+        <v>444.3</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>261.3</v>
+        <v>279.1</v>
       </c>
     </row>
     <row r="16">
@@ -846,28 +846,28 @@
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>1506.9</v>
+        <v>1510.4</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>491.4</v>
+        <v>481.8</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>2243.7</v>
+        <v>2246.7</v>
       </c>
       <c r="G16" s="6" t="n">
-        <v>828.6</v>
+        <v>812</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>1562.7</v>
+        <v>1553.6</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>631.9</v>
+        <v>620.8</v>
       </c>
       <c r="J16" s="6" t="n">
-        <v>736.8</v>
+        <v>736.3</v>
       </c>
     </row>
     <row r="17">
@@ -882,28 +882,28 @@
         </is>
       </c>
       <c r="C17" s="7" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D17" s="7" t="n">
-        <v>2966.9</v>
+        <v>2962.7</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>537.3</v>
+        <v>526.9</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>3329</v>
+        <v>3362.5</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>660.3</v>
+        <v>669.1</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>2639.4</v>
+        <v>2654.8</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>440.4</v>
+        <v>438.5</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>362.1</v>
+        <v>399.8</v>
       </c>
     </row>
     <row r="18">
@@ -918,28 +918,28 @@
         </is>
       </c>
       <c r="C18" s="7" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D18" s="7" t="n">
-        <v>2860.8</v>
+        <v>2848.4</v>
       </c>
       <c r="E18" s="7" t="n">
-        <v>504.2</v>
+        <v>498.1</v>
       </c>
       <c r="F18" s="7" t="n">
-        <v>4022.7</v>
+        <v>4015.6</v>
       </c>
       <c r="G18" s="7" t="n">
-        <v>1046.4</v>
+        <v>1025.9</v>
       </c>
       <c r="H18" s="7" t="n">
-        <v>3254</v>
+        <v>3233.2</v>
       </c>
       <c r="I18" s="7" t="n">
-        <v>891.5</v>
+        <v>879.9</v>
       </c>
       <c r="J18" s="7" t="n">
-        <v>1161.9</v>
+        <v>1167.2</v>
       </c>
     </row>
     <row r="19"/>
@@ -990,19 +990,19 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C23" s="5" t="n">
-        <v>91.59999999999999</v>
+        <v>91.7</v>
       </c>
       <c r="D23" s="5" t="n">
-        <v>92.2</v>
+        <v>92.5</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>93.3</v>
+        <v>93.2</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>92.40000000000001</v>
+        <v>92.5</v>
       </c>
     </row>
     <row r="24">
@@ -1012,19 +1012,19 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C24" s="6" t="n">
-        <v>93.8</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="D24" s="6" t="n">
-        <v>95.7</v>
+        <v>95.8</v>
       </c>
       <c r="E24" s="6" t="n">
         <v>94.5</v>
       </c>
       <c r="F24" s="6" t="n">
-        <v>94.5</v>
+        <v>94.59999999999999</v>
       </c>
     </row>
     <row r="25">
@@ -1034,16 +1034,16 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C25" s="7" t="n">
-        <v>89.3</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="D25" s="7" t="n">
-        <v>88.7</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>92.2</v>
+        <v>91.8</v>
       </c>
       <c r="F25" s="7" t="n">
         <v>90.3</v>
@@ -2345,6 +2345,56 @@
         <v>200.3</v>
       </c>
     </row>
+    <row r="80">
+      <c r="A80" s="7" t="n">
+        <v>74</v>
+      </c>
+      <c r="B80" s="7" t="inlineStr">
+        <is>
+          <t>ODOR</t>
+        </is>
+      </c>
+      <c r="C80" s="7" t="n">
+        <v>2669.14</v>
+      </c>
+      <c r="D80" s="7" t="n">
+        <v>4108.92</v>
+      </c>
+      <c r="E80" s="7" t="n">
+        <v>1439.8</v>
+      </c>
+      <c r="F80" s="7" t="n">
+        <v>2876.15</v>
+      </c>
+      <c r="G80" s="7" t="n">
+        <v>-207</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="6" t="n">
+        <v>75</v>
+      </c>
+      <c r="B81" s="6" t="inlineStr">
+        <is>
+          <t>PITCH</t>
+        </is>
+      </c>
+      <c r="C81" s="6" t="n">
+        <v>1621.38</v>
+      </c>
+      <c r="D81" s="6" t="n">
+        <v>2340.17</v>
+      </c>
+      <c r="E81" s="6" t="n">
+        <v>718.8</v>
+      </c>
+      <c r="F81" s="6" t="n">
+        <v>1506.3</v>
+      </c>
+      <c r="G81" s="6" t="n">
+        <v>115.1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>